<commit_message>
edit specification. add camera kreplenie
</commit_message>
<xml_diff>
--- a/спецификация.xlsx
+++ b/спецификация.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Herobib\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\всячена\project1 SUAI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4BC3F76-8B2B-4BFC-9556-5F8929D11B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA28C24A-91D0-40C8-BA8A-9BA72B234AB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{B57F1A92-7989-416A-991C-01B5D47EEC68}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="47">
   <si>
     <t>номер</t>
   </si>
@@ -106,6 +106,78 @@
   </si>
   <si>
     <t>переходник type-c to провод камеры</t>
+  </si>
+  <si>
+    <t>Dc-Dc преобразователь</t>
+  </si>
+  <si>
+    <t>Статус</t>
+  </si>
+  <si>
+    <t>дата</t>
+  </si>
+  <si>
+    <t>штырьевой разъем мама 2.54мм</t>
+  </si>
+  <si>
+    <t>48+запас</t>
+  </si>
+  <si>
+    <t>Получено</t>
+  </si>
+  <si>
+    <t>Куплен за свой счет</t>
+  </si>
+  <si>
+    <t>раньше</t>
+  </si>
+  <si>
+    <t>частично</t>
+  </si>
+  <si>
+    <t>Цена</t>
+  </si>
+  <si>
+    <t>ссылка</t>
+  </si>
+  <si>
+    <t>https://www.chipdip.ru/product/fc1-5211-tbh-18650-1a-p-batareynyy-otsek-1x18650-kls-9000296084</t>
+  </si>
+  <si>
+    <t>https://roboshop.spb.ru/modules/drajvery/drajvery-dvigatelej/l9110s-board</t>
+  </si>
+  <si>
+    <t>https://3drob.ru/arduino_datchiki_i_sensory/datchiki_priblizheniya/datchik_skorosti_opticheskiy_shelevoy_na_lm393</t>
+  </si>
+  <si>
+    <t>https://market.yandex.ru/card/10-sht-komplekt-koles-opticheskogo-enkodera-20cpr--6-mm-otverstiye-vala-povorotnyy-datchik-skorosti-disk-dlya-dvigatelya-postoyannogo-tokarobototekhnikiarduino/4331264543?ogV=345&amp;do-waremd5=yj24Glh-hyd8smNMjP6FmA&amp;cpc=bUEB-hf3wJN0F7ibQOLauTutREE6c9moH4YI_nvu3zj2rh9cZwGw0f8Q9aoZgfYP-ihB_3jBVhfwRqk64Z2t6hrcmVycipX26-3CaAtkvjiTP5A51bipcshbzHHUmt6g5gQGybEyfK8LUm4otvCC0aiSSPVIX3Pph7ZmyNxFAsycTXNxptf4nXulAMGNtEQ0yI3cTfpd5vYO9IhwR2PRJBi-634QrOpIjyEahvOys9USDJz2hqPChJe-vbVbCNNW706CFaZMYFXmYEvl84qv5rIB-VEL5qWp8ZMx5Ukvf7r9k3xKM6iYpxapsvxt_hD6i7CqGt8zrhxvAnf47P8QMqiOTcoJiPZpflVqc_uDgChLClD1f-xHqvA1CBYg7APjw8A-fUvceShVFJlqYiDCI24NlbzyLV7ZQ8rcfX_FH6BH8S5UXr-3wL3pEG23_8i1IA5_hhe0szBmEDKnpdE0BGlDHzc-A3yQ&amp;cc=CiA3MmEwMGYxZmFiZGYwMDExNDZjMmI1ZjVkZDM1OGJlMhAHgH3m7QY%2C&amp;resale_goods=resale_new&amp;hid=75685598&amp;nid=75685603&amp;show-uid=17906791142352336055206002&amp;showUid=17906791142352336055206002&amp;from-show-uid=17906791142352336055206002&amp;cpa=1&amp;bp_ao=12</t>
+  </si>
+  <si>
+    <t>https://www.ozon.ru/product/motor-s-reduktorom-dlya-arduino-robota-2-vyhodnyh-vala-1210887588/?at=1gan1TEXc31e8fqDxxxw9Pr-OFCRAK93&amp;sh=5HC01Aw0GQ</t>
+  </si>
+  <si>
+    <t>https://roboshop.spb.ru/radio/razieemy/shtyrkovye-razieemy/pls2-40-black</t>
+  </si>
+  <si>
+    <t>https://roboshop.spb.ru/radio/razieemy/shtyrkovye-razieemy/pbs-40-ds1023-1x40</t>
+  </si>
+  <si>
+    <t>https://www.ozon.ru/product/nabor-magnitov-silnyy-disk-5h3-mm-40sht-n52-5306461446/?at=1gan1YdLEsQweCi3tchBqCOLbQydT1Fi&amp;sh=5HC01Gy94w</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>болт М4*30</t>
+  </si>
+  <si>
+    <t>https://amperkot.ru/products/plata_razrabotchika_weact_esp32s3_n8r8_esp32s3devkitc1/40123550.html?srsltid=AU7gw4UGQq1VBnlcL9EYO8qOD0ERM3p0aPSOu4AV6okmYXuJit5zn0k2</t>
+  </si>
+  <si>
+    <t>https://www.ozon.ru/product/otg-perehodnik-s-type-c-na-usb-2923349978/?at=1gen1RKpZQJbx4HHu3buOqzQ7tuARzQp&amp;sh=5HC01Gy94w</t>
+  </si>
+  <si>
+    <t>ИТОГО</t>
   </si>
 </sst>
 </file>
@@ -130,7 +202,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -153,14 +225,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -475,19 +560,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{954E6C6C-EE81-407A-A1F1-5D1C8E4B4958}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="29" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,8 +585,23 @@
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -508,8 +611,17 @@
       <c r="C3" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1">
+        <v>64</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -519,8 +631,17 @@
       <c r="C4" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
+      <c r="F4" s="1"/>
+      <c r="G4" s="1">
+        <v>90</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -530,8 +651,17 @@
       <c r="C5" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+      <c r="F5" s="1"/>
+      <c r="G5" s="1">
+        <v>90</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -541,8 +671,23 @@
       <c r="C6" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="4">
+        <v>46287</v>
+      </c>
+      <c r="F6" s="1">
+        <v>2</v>
+      </c>
+      <c r="G6" s="2">
+        <v>75</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -552,8 +697,23 @@
       <c r="C7" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E7" s="4">
+        <v>46294</v>
+      </c>
+      <c r="F7" s="1">
+        <v>1</v>
+      </c>
+      <c r="G7" s="2">
+        <v>175</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -563,159 +723,361 @@
       <c r="C8" s="1">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D8" s="1"/>
+      <c r="E8" s="1"/>
+      <c r="F8" s="1"/>
+      <c r="G8" s="2">
+        <v>35</v>
+      </c>
+      <c r="H8" s="1"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="1">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
+      <c r="C9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="4">
+        <v>46287</v>
+      </c>
+      <c r="F9" s="1">
+        <v>480</v>
+      </c>
+      <c r="G9" s="2">
+        <v>17</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C10" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
+      <c r="F10" s="1"/>
+      <c r="G10" s="1">
+        <v>14</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C11" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+      <c r="H11" s="1"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C12" s="1">
         <v>10</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1">
+        <v>240</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" s="1"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14" s="1"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C15" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" s="1">
         <v>2</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D16" s="1"/>
+      <c r="E16" s="1"/>
+      <c r="F16" s="1"/>
+      <c r="G16" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C17" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17" s="1"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="1"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C19" s="1">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+      <c r="D19" s="1"/>
+      <c r="E19" s="1"/>
+      <c r="F19" s="1"/>
+      <c r="G19" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H19" s="1"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C20" s="1">
+        <v>8</v>
+      </c>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
+      <c r="G20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20" s="1"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="2">
-        <v>19</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="1">
+        <v>1</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E21" s="4">
+        <v>46287</v>
+      </c>
+      <c r="F21" s="1">
+        <v>1</v>
+      </c>
+      <c r="G21" s="2">
+        <v>990</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="2">
-        <v>20</v>
-      </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2">
+        <v>1</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" s="4">
+        <v>38989</v>
+      </c>
+      <c r="F22" s="1">
+        <v>1</v>
+      </c>
+      <c r="G22" s="2">
+        <v>600</v>
+      </c>
+      <c r="H22" s="1"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="2">
-        <v>1</v>
+      <c r="C23" s="2">
+        <v>1</v>
+      </c>
+      <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
+      <c r="F23" s="1"/>
+      <c r="G23" s="1">
+        <v>80</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>22</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" s="2">
+        <v>1</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F24" s="1">
+        <v>1</v>
+      </c>
+      <c r="G24" s="1">
+        <v>130</v>
+      </c>
+      <c r="H24" s="1"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C25" s="2">
+        <v>1</v>
+      </c>
+      <c r="D25" s="1"/>
+      <c r="E25" s="1"/>
+      <c r="F25" s="1"/>
+      <c r="G25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="H25" s="1"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="F26" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26">
+        <f>G3*C3+G4*C4+G5*C5+G6*C6+G7*C7+G8+G9*12+G10*12+G12+G21+G22+G23+G24</f>
+        <v>3345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>